<commit_message>
added vector IMP prefetcher with gretch-style OoO pattern detection
</commit_message>
<xml_diff>
--- a/tsvc_results/prefetcher_params.xlsx
+++ b/tsvc_results/prefetcher_params.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\parkw\gem5\tsvc_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB327A4-6D34-4C3F-9E51-FAC5E7B36920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146A23A6-F767-457C-A5B3-92728EB65432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefetcher Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="Base" sheetId="2" r:id="rId2"/>
     <sheet name="Stride" sheetId="3" r:id="rId3"/>
     <sheet name="IMP" sheetId="4" r:id="rId4"/>
-    <sheet name="ISB" sheetId="5" r:id="rId5"/>
-    <sheet name="STeMS" sheetId="6" r:id="rId6"/>
+    <sheet name="VIMP" sheetId="7" r:id="rId5"/>
+    <sheet name="ISB" sheetId="5" r:id="rId6"/>
+    <sheet name="STeMS" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1455" uniqueCount="100">
   <si>
     <t>Kernel</t>
   </si>
@@ -294,13 +317,59 @@
   <si>
     <t>4 KiB</t>
   </si>
+  <si>
+    <t>Checksum</t>
+  </si>
+  <si>
+    <t>indirect_delta</t>
+  </si>
+  <si>
+    <t>ipd_indices_per_chunk</t>
+  </si>
+  <si>
+    <t>PageRank</t>
+  </si>
+  <si>
+    <t>BFSCC</t>
+  </si>
+  <si>
+    <t>CF</t>
+  </si>
+  <si>
+    <t>Rounds</t>
+  </si>
+  <si>
+    <t>Input Graph</t>
+  </si>
+  <si>
+    <t>rMatGraph_J_5_100</t>
+  </si>
+  <si>
+    <t>sum = 0.980078125 max = 0.0213933138716</t>
+  </si>
+  <si>
+    <t>components = 4 labelSum = 46</t>
+  </si>
+  <si>
+    <t>For multiple rounds, we take the last round's stats</t>
+  </si>
+  <si>
+    <t>rMatGraph_WJ_5_100</t>
+  </si>
+  <si>
+    <t>latentSum = 1279.98837849</t>
+  </si>
+  <si>
+    <t>spmv</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -366,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -390,6 +459,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1013,20 +1084,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.36328125" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.90625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="37.08984375" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1045,14 +1120,17 @@
       <c r="F1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="7" t="s">
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1072,14 +1150,17 @@
         <f t="array" ref="F2:F25">D2:D25 / E2:E25</f>
         <v>0.16267327051104749</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="8">
         <v>0.64221499999999998</v>
       </c>
       <c r="H2">
         <v>0.21</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" s="14">
+        <v>30720</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1098,14 +1179,17 @@
       <c r="F3" s="8">
         <v>0.14366563668889251</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="8">
         <v>0.69885399999999998</v>
       </c>
       <c r="H3">
         <v>0.22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1124,14 +1208,17 @@
       <c r="F4" s="8">
         <v>0.12642380708055412</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="8">
         <v>0.62368400000000002</v>
       </c>
       <c r="H4">
         <v>-0.28999999999999998</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" s="14">
+        <v>15368.869140999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1150,14 +1237,17 @@
       <c r="F5" s="8">
         <v>7.5995864769152932E-2</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="8">
         <v>0.64485300000000001</v>
       </c>
       <c r="H5">
         <v>0.27</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1176,14 +1266,17 @@
       <c r="F6" s="8">
         <v>0.16322039818372336</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="8">
         <v>0.690052</v>
       </c>
       <c r="H6">
         <v>0.22</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6" s="14">
+        <v>15360</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1202,14 +1295,17 @@
       <c r="F7" s="8">
         <v>0.17554185722807716</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="8">
         <v>0.65839099999999995</v>
       </c>
       <c r="H7">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I7" s="14">
+        <v>1.0386359999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1228,14 +1324,17 @@
       <c r="F8" s="8">
         <v>0.42226707029936089</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="8">
         <v>6.8060000000000004E-3</v>
       </c>
       <c r="H8">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8" s="14">
+        <v>0.75323300000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1254,14 +1353,17 @@
       <c r="F9" s="8">
         <v>0.21707021791767556</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="8">
         <v>0.51293900000000003</v>
       </c>
       <c r="H9">
         <v>0.19</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" s="14">
+        <v>15362.205078000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1280,14 +1382,17 @@
       <c r="F10" s="8">
         <v>0.21753013210758085</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="8">
         <v>0.62556400000000001</v>
       </c>
       <c r="H10">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10" s="14">
+        <v>92160</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1306,14 +1411,17 @@
       <c r="F11" s="8">
         <v>0.14264892351534006</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="8">
         <v>0.69887500000000002</v>
       </c>
       <c r="H11">
         <v>0.74</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1332,14 +1440,17 @@
       <c r="F12" s="8">
         <v>0.1252319491979712</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="8">
         <v>0.62331599999999998</v>
       </c>
       <c r="H12">
         <v>0.68</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I12" s="14">
+        <v>15409.833984000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1358,14 +1469,17 @@
       <c r="F13" s="8">
         <v>7.5146143275641897E-2</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="8">
         <v>0.644841</v>
       </c>
       <c r="H13">
         <v>1.07</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I13" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1384,14 +1498,17 @@
       <c r="F14" s="8">
         <v>0.16211845278693826</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="8">
         <v>0.69004200000000004</v>
       </c>
       <c r="H14">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I14" s="14">
+        <v>15360</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1410,14 +1527,17 @@
       <c r="F15" s="8">
         <v>0.17452886808306325</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="8">
         <v>0.65839099999999995</v>
       </c>
       <c r="H15">
         <v>0.68</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15" s="14">
+        <v>1.0386359999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1436,14 +1556,17 @@
       <c r="F16" s="8">
         <v>0.42660644913311463</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="8">
         <v>1.361E-3</v>
       </c>
       <c r="H16">
         <v>0.49</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I16" s="14">
+        <v>0.75323300000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1462,14 +1585,17 @@
       <c r="F17" s="8">
         <v>0.2169980443285528</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="8">
         <v>0.51282899999999998</v>
       </c>
       <c r="H17">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17" s="14">
+        <v>15362.205078000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1488,14 +1614,17 @@
       <c r="F18" s="8">
         <v>0.22692711364917573</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="8">
         <v>0.62231300000000001</v>
       </c>
       <c r="H18">
         <v>1.36</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I18" s="14">
+        <v>168960</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1514,14 +1643,17 @@
       <c r="F19" s="8">
         <v>0.14250771726050332</v>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="8">
         <v>0.69886499999999996</v>
       </c>
       <c r="H19">
         <v>1.53</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I19" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1540,14 +1672,17 @@
       <c r="F20" s="8">
         <v>0.12512685727653339</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="8">
         <v>0.62324400000000002</v>
       </c>
       <c r="H20">
         <v>1.37</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I20" s="14">
+        <v>15462.979492</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -1566,14 +1701,17 @@
       <c r="F21" s="8">
         <v>7.5034486417657045E-2</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G21" s="8">
         <v>0.644868</v>
       </c>
       <c r="H21">
         <v>2.15</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I21" s="14">
+        <v>15361.640625</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -1592,14 +1730,17 @@
       <c r="F22" s="8">
         <v>0.16200185161065486</v>
       </c>
-      <c r="G22" s="12">
+      <c r="G22" s="8">
         <v>0.69004699999999997</v>
       </c>
       <c r="H22">
         <v>1.51</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I22" s="14">
+        <v>15360</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1618,14 +1759,17 @@
       <c r="F23" s="8">
         <v>0.17444561943216047</v>
       </c>
-      <c r="G23" s="12">
+      <c r="G23" s="8">
         <v>0.65839099999999995</v>
       </c>
       <c r="H23">
         <v>1.33</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I23" s="14">
+        <v>1.0386359999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -1644,14 +1788,17 @@
       <c r="F24" s="8">
         <v>0.42686608217294136</v>
       </c>
-      <c r="G24" s="12">
+      <c r="G24" s="8">
         <v>6.8099999999999996E-4</v>
       </c>
       <c r="H24">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I24" s="14">
+        <v>0.75323300000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -1670,11 +1817,351 @@
       <c r="F25" s="8">
         <v>0.21690726694396867</v>
       </c>
-      <c r="G25" s="12">
+      <c r="G25" s="8">
         <v>0.51319099999999995</v>
       </c>
       <c r="H25">
         <v>1.44</v>
+      </c>
+      <c r="I25" s="14">
+        <v>15362.205078000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29">
+        <v>512923</v>
+      </c>
+      <c r="E29">
+        <v>349893</v>
+      </c>
+      <c r="F29" s="8" cm="1">
+        <f t="array" ref="F29:F37" xml:space="preserve"> D29:D37 / E29:E37</f>
+        <v>1.4659424452618373</v>
+      </c>
+      <c r="G29" s="8">
+        <v>0.67671700000000001</v>
+      </c>
+      <c r="H29" s="8">
+        <v>2.06</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="M29" s="10"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30">
+        <v>34695</v>
+      </c>
+      <c r="E30">
+        <v>30188</v>
+      </c>
+      <c r="F30" s="8">
+        <v>1.1492977341990194</v>
+      </c>
+      <c r="G30" s="8">
+        <v>0.76190500000000005</v>
+      </c>
+      <c r="H30">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="M30" s="10"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31">
+        <v>474041</v>
+      </c>
+      <c r="E31">
+        <v>633253</v>
+      </c>
+      <c r="F31" s="8">
+        <v>0.74858074103083605</v>
+      </c>
+      <c r="G31" s="8">
+        <v>8.1767000000000006E-2</v>
+      </c>
+      <c r="H31" s="8">
+        <v>2.44</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="M31" s="10"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32">
+        <v>5</v>
+      </c>
+      <c r="C32" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32">
+        <v>512923</v>
+      </c>
+      <c r="E32">
+        <v>347795</v>
+      </c>
+      <c r="F32" s="8">
+        <v>1.4747854339481592</v>
+      </c>
+      <c r="G32" s="8">
+        <v>0.67783400000000005</v>
+      </c>
+      <c r="H32" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>93</v>
+      </c>
+      <c r="D33">
+        <v>34695</v>
+      </c>
+      <c r="E33">
+        <v>28737</v>
+      </c>
+      <c r="F33" s="8">
+        <v>1.2073285311619166</v>
+      </c>
+      <c r="G33" s="8">
+        <v>0.76190500000000005</v>
+      </c>
+      <c r="H33">
+        <v>0.27</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34">
+        <v>474041</v>
+      </c>
+      <c r="E34">
+        <v>631366</v>
+      </c>
+      <c r="F34" s="8">
+        <v>0.75081806749175595</v>
+      </c>
+      <c r="G34" s="8">
+        <v>8.1766000000000005E-2</v>
+      </c>
+      <c r="H34">
+        <v>3.62</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35">
+        <v>10</v>
+      </c>
+      <c r="C35" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35">
+        <v>512923</v>
+      </c>
+      <c r="E35">
+        <v>347851</v>
+      </c>
+      <c r="F35" s="8">
+        <v>1.4745480104987481</v>
+      </c>
+      <c r="G35" s="8">
+        <v>0.67688000000000004</v>
+      </c>
+      <c r="H35">
+        <v>2.29</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>89</v>
+      </c>
+      <c r="B36">
+        <v>10</v>
+      </c>
+      <c r="C36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36">
+        <v>34695</v>
+      </c>
+      <c r="E36">
+        <v>27792</v>
+      </c>
+      <c r="F36" s="8">
+        <v>1.248380829015544</v>
+      </c>
+      <c r="G36" s="8">
+        <v>0.78</v>
+      </c>
+      <c r="H36">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37">
+        <v>10</v>
+      </c>
+      <c r="C37" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37">
+        <v>474041</v>
+      </c>
+      <c r="E37">
+        <v>631644</v>
+      </c>
+      <c r="F37" s="8">
+        <v>0.7504876164421731</v>
+      </c>
+      <c r="G37" s="8">
+        <v>8.1848000000000004E-2</v>
+      </c>
+      <c r="H37">
+        <v>2.52</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I44"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1684,19 +2171,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M193"/>
+  <dimension ref="A1:O204"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.36328125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.90625" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.1796875" style="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.81640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.81640625" style="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.54296875" style="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16.81640625" style="10" bestFit="1" customWidth="1"/>
@@ -9576,7 +10063,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>21</v>
       </c>
@@ -9616,6 +10103,292 @@
       <c r="M193">
         <v>1.47</v>
       </c>
+    </row>
+    <row r="195" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A195" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C195" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D195" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E195" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F195" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G195" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H195" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I195" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J195" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K195"/>
+      <c r="M195"/>
+    </row>
+    <row r="196" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>88</v>
+      </c>
+      <c r="B196">
+        <v>1</v>
+      </c>
+      <c r="C196" t="s">
+        <v>93</v>
+      </c>
+      <c r="D196">
+        <v>4</v>
+      </c>
+      <c r="E196">
+        <v>0</v>
+      </c>
+      <c r="F196">
+        <v>512923</v>
+      </c>
+      <c r="H196" s="8" t="e" cm="1">
+        <f t="array" ref="H196:H204" xml:space="preserve"> F196:F204 / G196:G204</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I196" s="8"/>
+      <c r="J196" s="8"/>
+      <c r="M196"/>
+    </row>
+    <row r="197" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A197" t="s">
+        <v>89</v>
+      </c>
+      <c r="B197">
+        <v>1</v>
+      </c>
+      <c r="C197" t="s">
+        <v>93</v>
+      </c>
+      <c r="D197">
+        <v>4</v>
+      </c>
+      <c r="E197">
+        <v>0</v>
+      </c>
+      <c r="F197">
+        <v>34695</v>
+      </c>
+      <c r="H197" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I197" s="8"/>
+      <c r="J197"/>
+      <c r="K197" s="14"/>
+      <c r="M197"/>
+    </row>
+    <row r="198" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A198" t="s">
+        <v>90</v>
+      </c>
+      <c r="B198">
+        <v>1</v>
+      </c>
+      <c r="C198" t="s">
+        <v>97</v>
+      </c>
+      <c r="D198">
+        <v>4</v>
+      </c>
+      <c r="E198">
+        <v>0</v>
+      </c>
+      <c r="F198">
+        <v>474041</v>
+      </c>
+      <c r="H198" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I198" s="8"/>
+      <c r="J198" s="8"/>
+      <c r="M198"/>
+    </row>
+    <row r="199" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A199" t="s">
+        <v>88</v>
+      </c>
+      <c r="B199">
+        <v>5</v>
+      </c>
+      <c r="C199" t="s">
+        <v>93</v>
+      </c>
+      <c r="D199">
+        <v>4</v>
+      </c>
+      <c r="E199">
+        <v>0</v>
+      </c>
+      <c r="F199">
+        <v>512923</v>
+      </c>
+      <c r="H199" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I199" s="8"/>
+      <c r="J199" s="8"/>
+      <c r="L199" s="12"/>
+      <c r="M199" s="12"/>
+      <c r="O199" s="10"/>
+    </row>
+    <row r="200" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A200" t="s">
+        <v>89</v>
+      </c>
+      <c r="B200">
+        <v>5</v>
+      </c>
+      <c r="C200" t="s">
+        <v>93</v>
+      </c>
+      <c r="D200">
+        <v>4</v>
+      </c>
+      <c r="E200">
+        <v>0</v>
+      </c>
+      <c r="F200">
+        <v>34695</v>
+      </c>
+      <c r="H200" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I200" s="8"/>
+      <c r="J200"/>
+      <c r="K200" s="14"/>
+      <c r="L200" s="12"/>
+      <c r="M200" s="12"/>
+      <c r="O200" s="10"/>
+    </row>
+    <row r="201" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A201" t="s">
+        <v>90</v>
+      </c>
+      <c r="B201">
+        <v>5</v>
+      </c>
+      <c r="C201" t="s">
+        <v>97</v>
+      </c>
+      <c r="D201">
+        <v>4</v>
+      </c>
+      <c r="E201">
+        <v>0</v>
+      </c>
+      <c r="F201">
+        <v>474041</v>
+      </c>
+      <c r="H201" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I201" s="8"/>
+      <c r="J201"/>
+      <c r="K201" s="14"/>
+      <c r="L201" s="12"/>
+      <c r="M201" s="12"/>
+      <c r="O201" s="10"/>
+    </row>
+    <row r="202" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A202" t="s">
+        <v>88</v>
+      </c>
+      <c r="B202">
+        <v>10</v>
+      </c>
+      <c r="C202" t="s">
+        <v>93</v>
+      </c>
+      <c r="D202">
+        <v>4</v>
+      </c>
+      <c r="E202">
+        <v>0</v>
+      </c>
+      <c r="F202">
+        <v>512923</v>
+      </c>
+      <c r="H202" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I202" s="8"/>
+      <c r="J202"/>
+      <c r="L202" s="12"/>
+      <c r="M202" s="12"/>
+      <c r="O202" s="10"/>
+    </row>
+    <row r="203" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A203" t="s">
+        <v>89</v>
+      </c>
+      <c r="B203">
+        <v>10</v>
+      </c>
+      <c r="C203" t="s">
+        <v>93</v>
+      </c>
+      <c r="D203">
+        <v>4</v>
+      </c>
+      <c r="E203">
+        <v>0</v>
+      </c>
+      <c r="F203">
+        <v>34695</v>
+      </c>
+      <c r="H203" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I203" s="8"/>
+      <c r="J203"/>
+      <c r="K203" s="14"/>
+      <c r="L203" s="12"/>
+      <c r="M203" s="12"/>
+      <c r="O203" s="10"/>
+    </row>
+    <row r="204" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A204" t="s">
+        <v>90</v>
+      </c>
+      <c r="B204">
+        <v>10</v>
+      </c>
+      <c r="C204" t="s">
+        <v>97</v>
+      </c>
+      <c r="D204">
+        <v>4</v>
+      </c>
+      <c r="E204">
+        <v>0</v>
+      </c>
+      <c r="F204">
+        <v>474041</v>
+      </c>
+      <c r="H204" s="8" t="e">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I204" s="8"/>
+      <c r="J204"/>
+      <c r="K204" s="14"/>
+      <c r="L204" s="12"/>
+      <c r="M204" s="12"/>
+      <c r="O204" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14609,6 +15382,2674 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2BB61EF-C124-47C3-8951-0338D3730893}">
+  <dimension ref="A1:P79"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>5058</v>
+      </c>
+      <c r="J2">
+        <v>30667</v>
+      </c>
+      <c r="K2" s="8" cm="1">
+        <f t="array" ref="K2:K73" xml:space="preserve"> I2:I73 / J2:J73</f>
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>4417</v>
+      </c>
+      <c r="J3">
+        <v>19283</v>
+      </c>
+      <c r="K3" s="8">
+        <v>0.22906186796660272</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>8</v>
+      </c>
+      <c r="I4">
+        <v>3696</v>
+      </c>
+      <c r="J4">
+        <v>18216</v>
+      </c>
+      <c r="K4" s="8">
+        <v>0.20289855072463769</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5">
+        <v>3455</v>
+      </c>
+      <c r="J5">
+        <v>32292</v>
+      </c>
+      <c r="K5" s="8">
+        <v>0.10699244394896569</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>4673</v>
+      </c>
+      <c r="J6">
+        <v>23397</v>
+      </c>
+      <c r="K6" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>4414</v>
+      </c>
+      <c r="J7">
+        <v>15939</v>
+      </c>
+      <c r="K7" s="8">
+        <v>0.27693079866992909</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8">
+        <v>6277</v>
+      </c>
+      <c r="J8">
+        <v>14936</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+      <c r="I9">
+        <v>5379</v>
+      </c>
+      <c r="J9">
+        <v>26608</v>
+      </c>
+      <c r="K9" s="8">
+        <v>0.20215724594107035</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <v>4</v>
+      </c>
+      <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
+        <v>5058</v>
+      </c>
+      <c r="J10">
+        <v>30667</v>
+      </c>
+      <c r="K10" s="8">
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>4</v>
+      </c>
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11">
+        <v>4417</v>
+      </c>
+      <c r="J11">
+        <v>19277</v>
+      </c>
+      <c r="K11" s="8">
+        <v>0.22913316387404678</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12">
+        <v>4</v>
+      </c>
+      <c r="H12">
+        <v>8</v>
+      </c>
+      <c r="I12">
+        <v>3696</v>
+      </c>
+      <c r="J12">
+        <v>18353</v>
+      </c>
+      <c r="K12" s="8">
+        <v>0.20138396992317331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13">
+        <v>8</v>
+      </c>
+      <c r="I13">
+        <v>3455</v>
+      </c>
+      <c r="J13">
+        <v>32572</v>
+      </c>
+      <c r="K13" s="8">
+        <v>0.10607270047893896</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <v>4</v>
+      </c>
+      <c r="H14">
+        <v>8</v>
+      </c>
+      <c r="I14">
+        <v>4673</v>
+      </c>
+      <c r="J14">
+        <v>23397</v>
+      </c>
+      <c r="K14" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>4</v>
+      </c>
+      <c r="G15">
+        <v>4</v>
+      </c>
+      <c r="H15">
+        <v>8</v>
+      </c>
+      <c r="I15">
+        <v>4414</v>
+      </c>
+      <c r="J15">
+        <v>16054</v>
+      </c>
+      <c r="K15" s="8">
+        <v>0.27494705369378347</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="I16">
+        <v>6277</v>
+      </c>
+      <c r="J16">
+        <v>14936</v>
+      </c>
+      <c r="K16" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17">
+        <v>8</v>
+      </c>
+      <c r="I17">
+        <v>5379</v>
+      </c>
+      <c r="J17">
+        <v>26606</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0.2021724423062467</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18">
+        <v>8</v>
+      </c>
+      <c r="I18">
+        <v>5058</v>
+      </c>
+      <c r="J18">
+        <v>30667</v>
+      </c>
+      <c r="K18" s="8">
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
+      <c r="G19">
+        <v>4</v>
+      </c>
+      <c r="H19">
+        <v>8</v>
+      </c>
+      <c r="I19">
+        <v>4417</v>
+      </c>
+      <c r="J19">
+        <v>19283</v>
+      </c>
+      <c r="K19" s="8">
+        <v>0.22906186796660272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
+        <v>4</v>
+      </c>
+      <c r="H20">
+        <v>8</v>
+      </c>
+      <c r="I20">
+        <v>3696</v>
+      </c>
+      <c r="J20">
+        <v>18216</v>
+      </c>
+      <c r="K20" s="8">
+        <v>0.20289855072463769</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21">
+        <v>8</v>
+      </c>
+      <c r="I21">
+        <v>3455</v>
+      </c>
+      <c r="J21">
+        <v>32292</v>
+      </c>
+      <c r="K21" s="8">
+        <v>0.10699244394896569</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>4673</v>
+      </c>
+      <c r="J22">
+        <v>23397</v>
+      </c>
+      <c r="K22" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>4</v>
+      </c>
+      <c r="G23">
+        <v>4</v>
+      </c>
+      <c r="H23">
+        <v>8</v>
+      </c>
+      <c r="I23">
+        <v>4414</v>
+      </c>
+      <c r="J23">
+        <v>15939</v>
+      </c>
+      <c r="K23" s="8">
+        <v>0.27693079866992909</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>4</v>
+      </c>
+      <c r="G24">
+        <v>4</v>
+      </c>
+      <c r="H24">
+        <v>8</v>
+      </c>
+      <c r="I24">
+        <v>6277</v>
+      </c>
+      <c r="J24">
+        <v>14936</v>
+      </c>
+      <c r="K24" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>4</v>
+      </c>
+      <c r="G25">
+        <v>4</v>
+      </c>
+      <c r="H25">
+        <v>8</v>
+      </c>
+      <c r="I25">
+        <v>5379</v>
+      </c>
+      <c r="J25">
+        <v>26608</v>
+      </c>
+      <c r="K25" s="8">
+        <v>0.20215724594107035</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>4</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+      <c r="G26">
+        <v>4</v>
+      </c>
+      <c r="H26">
+        <v>8</v>
+      </c>
+      <c r="I26">
+        <v>5058</v>
+      </c>
+      <c r="J26">
+        <v>30667</v>
+      </c>
+      <c r="K26" s="8">
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>15</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>4</v>
+      </c>
+      <c r="F27">
+        <v>4</v>
+      </c>
+      <c r="G27">
+        <v>4</v>
+      </c>
+      <c r="H27">
+        <v>8</v>
+      </c>
+      <c r="I27">
+        <v>4417</v>
+      </c>
+      <c r="J27">
+        <v>21111</v>
+      </c>
+      <c r="K27" s="8">
+        <v>0.20922741698640518</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28">
+        <v>4</v>
+      </c>
+      <c r="G28">
+        <v>4</v>
+      </c>
+      <c r="H28">
+        <v>8</v>
+      </c>
+      <c r="I28">
+        <v>3696</v>
+      </c>
+      <c r="J28">
+        <v>18737</v>
+      </c>
+      <c r="K28" s="8">
+        <v>0.19725676469018519</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>4</v>
+      </c>
+      <c r="F29">
+        <v>4</v>
+      </c>
+      <c r="G29">
+        <v>4</v>
+      </c>
+      <c r="H29">
+        <v>8</v>
+      </c>
+      <c r="I29">
+        <v>3455</v>
+      </c>
+      <c r="J29">
+        <v>33404</v>
+      </c>
+      <c r="K29" s="8">
+        <v>0.1034307268590588</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>4</v>
+      </c>
+      <c r="F30">
+        <v>4</v>
+      </c>
+      <c r="G30">
+        <v>4</v>
+      </c>
+      <c r="H30">
+        <v>8</v>
+      </c>
+      <c r="I30">
+        <v>4673</v>
+      </c>
+      <c r="J30">
+        <v>23397</v>
+      </c>
+      <c r="K30" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>4</v>
+      </c>
+      <c r="F31">
+        <v>4</v>
+      </c>
+      <c r="G31">
+        <v>4</v>
+      </c>
+      <c r="H31">
+        <v>8</v>
+      </c>
+      <c r="I31">
+        <v>4414</v>
+      </c>
+      <c r="J31">
+        <v>16035</v>
+      </c>
+      <c r="K31" s="8">
+        <v>0.27527284066105395</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>4</v>
+      </c>
+      <c r="F32">
+        <v>4</v>
+      </c>
+      <c r="G32">
+        <v>4</v>
+      </c>
+      <c r="H32">
+        <v>8</v>
+      </c>
+      <c r="I32">
+        <v>6277</v>
+      </c>
+      <c r="J32">
+        <v>14936</v>
+      </c>
+      <c r="K32" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>4</v>
+      </c>
+      <c r="F33">
+        <v>4</v>
+      </c>
+      <c r="G33">
+        <v>4</v>
+      </c>
+      <c r="H33">
+        <v>8</v>
+      </c>
+      <c r="I33">
+        <v>5379</v>
+      </c>
+      <c r="J33">
+        <v>26606</v>
+      </c>
+      <c r="K33" s="8">
+        <v>0.2021724423062467</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+      <c r="F34">
+        <v>2</v>
+      </c>
+      <c r="G34">
+        <v>4</v>
+      </c>
+      <c r="H34">
+        <v>8</v>
+      </c>
+      <c r="I34">
+        <v>5058</v>
+      </c>
+      <c r="J34">
+        <v>25899</v>
+      </c>
+      <c r="K34" s="8">
+        <v>0.19529711571875363</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>2</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+      <c r="G35">
+        <v>4</v>
+      </c>
+      <c r="H35">
+        <v>8</v>
+      </c>
+      <c r="I35">
+        <v>4417</v>
+      </c>
+      <c r="J35">
+        <v>19563</v>
+      </c>
+      <c r="K35" s="8">
+        <v>0.22578336655932116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>4</v>
+      </c>
+      <c r="H36">
+        <v>8</v>
+      </c>
+      <c r="I36">
+        <v>3696</v>
+      </c>
+      <c r="J36">
+        <v>18080</v>
+      </c>
+      <c r="K36" s="8">
+        <v>0.20442477876106194</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37">
+        <v>4</v>
+      </c>
+      <c r="H37">
+        <v>8</v>
+      </c>
+      <c r="I37">
+        <v>3455</v>
+      </c>
+      <c r="J37">
+        <v>36640</v>
+      </c>
+      <c r="K37" s="8">
+        <v>9.4295851528384281E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>4</v>
+      </c>
+      <c r="H38">
+        <v>8</v>
+      </c>
+      <c r="I38">
+        <v>4673</v>
+      </c>
+      <c r="J38">
+        <v>23274</v>
+      </c>
+      <c r="K38" s="8">
+        <v>0.20078198848500473</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+      <c r="F39">
+        <v>2</v>
+      </c>
+      <c r="G39">
+        <v>4</v>
+      </c>
+      <c r="H39">
+        <v>8</v>
+      </c>
+      <c r="I39">
+        <v>4414</v>
+      </c>
+      <c r="J39">
+        <v>21038</v>
+      </c>
+      <c r="K39" s="8">
+        <v>0.20981081851887062</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40">
+        <v>4</v>
+      </c>
+      <c r="H40">
+        <v>8</v>
+      </c>
+      <c r="I40">
+        <v>6277</v>
+      </c>
+      <c r="J40">
+        <v>14911</v>
+      </c>
+      <c r="K40" s="8">
+        <v>0.42096438870632419</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>21</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+      <c r="C41" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41">
+        <v>4</v>
+      </c>
+      <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>5379</v>
+      </c>
+      <c r="J41">
+        <v>26632</v>
+      </c>
+      <c r="K41" s="8">
+        <v>0.20197506758786421</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>4</v>
+      </c>
+      <c r="G42">
+        <v>8</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
+      </c>
+      <c r="I42">
+        <v>5058</v>
+      </c>
+      <c r="J42">
+        <v>31296</v>
+      </c>
+      <c r="K42" s="8">
+        <v>0.1616180981595092</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>4</v>
+      </c>
+      <c r="G43">
+        <v>8</v>
+      </c>
+      <c r="H43">
+        <v>8</v>
+      </c>
+      <c r="I43">
+        <v>4417</v>
+      </c>
+      <c r="J43">
+        <v>18993</v>
+      </c>
+      <c r="K43" s="8">
+        <v>0.23255936397620175</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>2</v>
+      </c>
+      <c r="F44">
+        <v>4</v>
+      </c>
+      <c r="G44">
+        <v>8</v>
+      </c>
+      <c r="H44">
+        <v>8</v>
+      </c>
+      <c r="I44">
+        <v>3696</v>
+      </c>
+      <c r="J44">
+        <v>19217</v>
+      </c>
+      <c r="K44" s="8">
+        <v>0.19232970807097882</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>4</v>
+      </c>
+      <c r="G45">
+        <v>8</v>
+      </c>
+      <c r="H45">
+        <v>8</v>
+      </c>
+      <c r="I45">
+        <v>3455</v>
+      </c>
+      <c r="J45">
+        <v>32334</v>
+      </c>
+      <c r="K45" s="8">
+        <v>0.106853466938826</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>2</v>
+      </c>
+      <c r="F46">
+        <v>4</v>
+      </c>
+      <c r="G46">
+        <v>8</v>
+      </c>
+      <c r="H46">
+        <v>8</v>
+      </c>
+      <c r="I46">
+        <v>4673</v>
+      </c>
+      <c r="J46">
+        <v>23847</v>
+      </c>
+      <c r="K46" s="8">
+        <v>0.19595756279615884</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>19</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <v>4</v>
+      </c>
+      <c r="G47">
+        <v>8</v>
+      </c>
+      <c r="H47">
+        <v>8</v>
+      </c>
+      <c r="I47">
+        <v>4414</v>
+      </c>
+      <c r="J47">
+        <v>15928</v>
+      </c>
+      <c r="K47" s="8">
+        <v>0.27712204922149675</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>2</v>
+      </c>
+      <c r="F48">
+        <v>4</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
+        <v>8</v>
+      </c>
+      <c r="I48">
+        <v>6277</v>
+      </c>
+      <c r="J48">
+        <v>14936</v>
+      </c>
+      <c r="K48" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>21</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>2</v>
+      </c>
+      <c r="F49">
+        <v>4</v>
+      </c>
+      <c r="G49">
+        <v>8</v>
+      </c>
+      <c r="H49">
+        <v>8</v>
+      </c>
+      <c r="I49">
+        <v>5379</v>
+      </c>
+      <c r="J49">
+        <v>26973</v>
+      </c>
+      <c r="K49" s="8">
+        <v>0.19942164386608832</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50">
+        <v>8</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <v>4</v>
+      </c>
+      <c r="G50">
+        <v>8</v>
+      </c>
+      <c r="H50">
+        <v>8</v>
+      </c>
+      <c r="I50">
+        <v>5058</v>
+      </c>
+      <c r="J50">
+        <v>31296</v>
+      </c>
+      <c r="K50" s="8">
+        <v>0.1616180981595092</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51">
+        <v>8</v>
+      </c>
+      <c r="E51">
+        <v>2</v>
+      </c>
+      <c r="F51">
+        <v>4</v>
+      </c>
+      <c r="G51">
+        <v>8</v>
+      </c>
+      <c r="H51">
+        <v>8</v>
+      </c>
+      <c r="I51">
+        <v>4417</v>
+      </c>
+      <c r="J51">
+        <v>18022</v>
+      </c>
+      <c r="K51" s="8">
+        <v>0.24508933525690824</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52">
+        <v>8</v>
+      </c>
+      <c r="E52">
+        <v>2</v>
+      </c>
+      <c r="F52">
+        <v>4</v>
+      </c>
+      <c r="G52">
+        <v>8</v>
+      </c>
+      <c r="H52">
+        <v>8</v>
+      </c>
+      <c r="I52">
+        <v>3696</v>
+      </c>
+      <c r="J52">
+        <v>18937</v>
+      </c>
+      <c r="K52" s="8">
+        <v>0.19517346992659873</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53">
+        <v>8</v>
+      </c>
+      <c r="E53">
+        <v>2</v>
+      </c>
+      <c r="F53">
+        <v>4</v>
+      </c>
+      <c r="G53">
+        <v>8</v>
+      </c>
+      <c r="H53">
+        <v>8</v>
+      </c>
+      <c r="I53">
+        <v>3455</v>
+      </c>
+      <c r="J53">
+        <v>32925</v>
+      </c>
+      <c r="K53" s="8">
+        <v>0.10493545937737282</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D54">
+        <v>8</v>
+      </c>
+      <c r="E54">
+        <v>2</v>
+      </c>
+      <c r="F54">
+        <v>4</v>
+      </c>
+      <c r="G54">
+        <v>8</v>
+      </c>
+      <c r="H54">
+        <v>8</v>
+      </c>
+      <c r="I54">
+        <v>4673</v>
+      </c>
+      <c r="J54">
+        <v>23847</v>
+      </c>
+      <c r="K54" s="8">
+        <v>0.19595756279615884</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" t="s">
+        <v>14</v>
+      </c>
+      <c r="D55">
+        <v>8</v>
+      </c>
+      <c r="E55">
+        <v>2</v>
+      </c>
+      <c r="F55">
+        <v>4</v>
+      </c>
+      <c r="G55">
+        <v>8</v>
+      </c>
+      <c r="H55">
+        <v>8</v>
+      </c>
+      <c r="I55">
+        <v>4414</v>
+      </c>
+      <c r="J55">
+        <v>16502</v>
+      </c>
+      <c r="K55" s="8">
+        <v>0.26748272936613743</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56">
+        <v>8</v>
+      </c>
+      <c r="E56">
+        <v>2</v>
+      </c>
+      <c r="F56">
+        <v>4</v>
+      </c>
+      <c r="G56">
+        <v>8</v>
+      </c>
+      <c r="H56">
+        <v>8</v>
+      </c>
+      <c r="I56">
+        <v>6277</v>
+      </c>
+      <c r="J56">
+        <v>14936</v>
+      </c>
+      <c r="K56" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>21</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57">
+        <v>8</v>
+      </c>
+      <c r="E57">
+        <v>2</v>
+      </c>
+      <c r="F57">
+        <v>4</v>
+      </c>
+      <c r="G57">
+        <v>8</v>
+      </c>
+      <c r="H57">
+        <v>8</v>
+      </c>
+      <c r="I57">
+        <v>5379</v>
+      </c>
+      <c r="J57">
+        <v>26979</v>
+      </c>
+      <c r="K57" s="8">
+        <v>0.19937729345046146</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>13</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>14</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>2</v>
+      </c>
+      <c r="F58">
+        <v>4</v>
+      </c>
+      <c r="G58">
+        <v>4</v>
+      </c>
+      <c r="H58">
+        <v>4</v>
+      </c>
+      <c r="I58">
+        <v>5058</v>
+      </c>
+      <c r="J58">
+        <v>30667</v>
+      </c>
+      <c r="K58" s="8">
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>2</v>
+      </c>
+      <c r="F59">
+        <v>4</v>
+      </c>
+      <c r="G59">
+        <v>4</v>
+      </c>
+      <c r="H59">
+        <v>4</v>
+      </c>
+      <c r="I59">
+        <v>4417</v>
+      </c>
+      <c r="J59">
+        <v>19600</v>
+      </c>
+      <c r="K59" s="8">
+        <v>0.22535714285714287</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>16</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>14</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>2</v>
+      </c>
+      <c r="F60">
+        <v>4</v>
+      </c>
+      <c r="G60">
+        <v>4</v>
+      </c>
+      <c r="H60">
+        <v>4</v>
+      </c>
+      <c r="I60">
+        <v>3696</v>
+      </c>
+      <c r="J60">
+        <v>22878</v>
+      </c>
+      <c r="K60" s="8">
+        <v>0.16155258326776817</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>17</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>2</v>
+      </c>
+      <c r="F61">
+        <v>4</v>
+      </c>
+      <c r="G61">
+        <v>4</v>
+      </c>
+      <c r="H61">
+        <v>4</v>
+      </c>
+      <c r="I61">
+        <v>3455</v>
+      </c>
+      <c r="J61">
+        <v>39402</v>
+      </c>
+      <c r="K61" s="8">
+        <v>8.7685904268818837E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>2</v>
+      </c>
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>4</v>
+      </c>
+      <c r="H62">
+        <v>4</v>
+      </c>
+      <c r="I62">
+        <v>4673</v>
+      </c>
+      <c r="J62">
+        <v>23397</v>
+      </c>
+      <c r="K62" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>2</v>
+      </c>
+      <c r="F63">
+        <v>4</v>
+      </c>
+      <c r="G63">
+        <v>4</v>
+      </c>
+      <c r="H63">
+        <v>4</v>
+      </c>
+      <c r="I63">
+        <v>4414</v>
+      </c>
+      <c r="J63">
+        <v>18827</v>
+      </c>
+      <c r="K63" s="8">
+        <v>0.23445052318478782</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>2</v>
+      </c>
+      <c r="F64">
+        <v>4</v>
+      </c>
+      <c r="G64">
+        <v>4</v>
+      </c>
+      <c r="H64">
+        <v>4</v>
+      </c>
+      <c r="I64">
+        <v>6277</v>
+      </c>
+      <c r="J64">
+        <v>14936</v>
+      </c>
+      <c r="K64" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>21</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" t="s">
+        <v>14</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>2</v>
+      </c>
+      <c r="F65">
+        <v>4</v>
+      </c>
+      <c r="G65">
+        <v>4</v>
+      </c>
+      <c r="H65">
+        <v>4</v>
+      </c>
+      <c r="I65">
+        <v>5379</v>
+      </c>
+      <c r="J65">
+        <v>26610</v>
+      </c>
+      <c r="K65" s="8">
+        <v>0.20214205186020293</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>2</v>
+      </c>
+      <c r="F66">
+        <v>4</v>
+      </c>
+      <c r="G66">
+        <v>4</v>
+      </c>
+      <c r="H66">
+        <v>16</v>
+      </c>
+      <c r="I66">
+        <v>5058</v>
+      </c>
+      <c r="J66">
+        <v>30667</v>
+      </c>
+      <c r="K66" s="8">
+        <v>0.16493298985880589</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>15</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>2</v>
+      </c>
+      <c r="F67">
+        <v>4</v>
+      </c>
+      <c r="G67">
+        <v>4</v>
+      </c>
+      <c r="H67">
+        <v>16</v>
+      </c>
+      <c r="I67">
+        <v>4417</v>
+      </c>
+      <c r="J67">
+        <v>19600</v>
+      </c>
+      <c r="K67" s="8">
+        <v>0.22535714285714287</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>16</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>2</v>
+      </c>
+      <c r="F68">
+        <v>4</v>
+      </c>
+      <c r="G68">
+        <v>4</v>
+      </c>
+      <c r="H68">
+        <v>16</v>
+      </c>
+      <c r="I68">
+        <v>3696</v>
+      </c>
+      <c r="J68">
+        <v>22868</v>
+      </c>
+      <c r="K68" s="8">
+        <v>0.16162322896624104</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>17</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>14</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>2</v>
+      </c>
+      <c r="F69">
+        <v>4</v>
+      </c>
+      <c r="G69">
+        <v>4</v>
+      </c>
+      <c r="H69">
+        <v>16</v>
+      </c>
+      <c r="I69">
+        <v>3455</v>
+      </c>
+      <c r="J69">
+        <v>39412</v>
+      </c>
+      <c r="K69" s="8">
+        <v>8.7663655739368726E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>18</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" t="s">
+        <v>14</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>2</v>
+      </c>
+      <c r="F70">
+        <v>4</v>
+      </c>
+      <c r="G70">
+        <v>4</v>
+      </c>
+      <c r="H70">
+        <v>16</v>
+      </c>
+      <c r="I70">
+        <v>4673</v>
+      </c>
+      <c r="J70">
+        <v>23397</v>
+      </c>
+      <c r="K70" s="8">
+        <v>0.19972646065734923</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>19</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>14</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>2</v>
+      </c>
+      <c r="F71">
+        <v>4</v>
+      </c>
+      <c r="G71">
+        <v>4</v>
+      </c>
+      <c r="H71">
+        <v>16</v>
+      </c>
+      <c r="I71">
+        <v>4414</v>
+      </c>
+      <c r="J71">
+        <v>21054</v>
+      </c>
+      <c r="K71" s="8">
+        <v>0.20965137266077705</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>20</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
+      <c r="F72">
+        <v>4</v>
+      </c>
+      <c r="G72">
+        <v>4</v>
+      </c>
+      <c r="H72">
+        <v>16</v>
+      </c>
+      <c r="I72">
+        <v>6277</v>
+      </c>
+      <c r="J72">
+        <v>14936</v>
+      </c>
+      <c r="K72" s="8">
+        <v>0.42025977504017142</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>21</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>14</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73">
+        <v>2</v>
+      </c>
+      <c r="F73">
+        <v>4</v>
+      </c>
+      <c r="G73">
+        <v>4</v>
+      </c>
+      <c r="H73">
+        <v>16</v>
+      </c>
+      <c r="I73">
+        <v>5379</v>
+      </c>
+      <c r="J73">
+        <v>26606</v>
+      </c>
+      <c r="K73" s="8">
+        <v>0.2021724423062467</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A76" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H76" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I76" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K76" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="L76" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>88</v>
+      </c>
+      <c r="H77" s="8"/>
+      <c r="I77" s="12"/>
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+      <c r="M77" s="10"/>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>89</v>
+      </c>
+      <c r="H78" s="8"/>
+      <c r="I78" s="12"/>
+      <c r="J78" s="12"/>
+      <c r="K78" s="12"/>
+      <c r="M78" s="10"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>90</v>
+      </c>
+      <c r="H79" s="8"/>
+      <c r="I79" s="12"/>
+      <c r="J79" s="12"/>
+      <c r="K79" s="12"/>
+      <c r="M79" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M97"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -18611,7 +22052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:M73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>